<commit_message>
changing the theme and setting up the args
</commit_message>
<xml_diff>
--- a/data/Brand Sheet.xlsx
+++ b/data/Brand Sheet.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t xml:space="preserve">COMPANY</t>
   </si>
@@ -31,40 +31,13 @@
     <t xml:space="preserve">Gmail</t>
   </si>
   <si>
-    <t xml:space="preserve">HERSAY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avishkar Sonawane</t>
-  </si>
-  <si>
-    <t xml:space="preserve">smahadik713@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Svarasya</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deepti Sehgal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@svarasya.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kzen Skincare</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preeti</t>
-  </si>
-  <si>
-    <t xml:space="preserve">preeti@kzenskincare.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OG  BEAUTY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Harshil Amrania</t>
-  </si>
-  <si>
-    <t xml:space="preserve">harshilamrania@gmail.com</t>
+    <t xml:space="preserve">WorkerSSal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Akram</t>
+  </si>
+  <si>
+    <t xml:space="preserve">akram.codes.it@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -276,9 +249,9 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:W6"/>
-  <sheetFormatPr defaultColWidth="12.640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.66015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.89"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.77"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26.03"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1021" style="0" width="11.52"/>
@@ -315,7 +288,7 @@
       <c r="V1" s="2"/>
       <c r="W1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -346,16 +319,10 @@
       <c r="V2" s="2"/>
       <c r="W2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>8</v>
-      </c>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="3"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
@@ -377,16 +344,10 @@
       <c r="V3" s="2"/>
       <c r="W3" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>11</v>
-      </c>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="4"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
@@ -408,16 +369,10 @@
       <c r="V4" s="2"/>
       <c r="W4" s="2"/>
     </row>
-    <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>14</v>
-      </c>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="3"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
@@ -439,16 +394,10 @@
       <c r="V5" s="2"/>
       <c r="W5" s="2"/>
     </row>
-    <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>8</v>
-      </c>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="3"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
@@ -472,11 +421,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" display="smahadik713@gmail.com"/>
-    <hyperlink ref="C3" r:id="rId2" display="contact@svarasya.com"/>
-    <hyperlink ref="C4" r:id="rId3" display="preeti@kzenskincare.com"/>
-    <hyperlink ref="C5" r:id="rId4" display="harshilamrania@gmail.com"/>
-    <hyperlink ref="C6" r:id="rId5" display="contact@svarasya.com"/>
+    <hyperlink ref="C2" r:id="rId1" display="akram.codes.it@gmail.com"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>